<commit_message>
Rate schedules: any rate can change over time
Emigration, fill rates, completion and external entrants accept a {year: value} path with linear interpolation, held flat outside the anchor years. Editable Year/Value tables in the sidebar, rate-path charts on the Sensitivity tab. All defaults remain constants, so published figures are unchanged (verified at 0.000000).

Also fixes a real non-determinism bug: the column-name matchers were Python sets, and where a sheet carried both sanctionedseats and totalapprovedseats the choice depended on set iteration order, which varies per process. B.Pharm 2024 read as 9,270 or 9,275 at random. Matchers are now ordered lists preferring sanctioned seats, since lateral-entry seats join in year two with a shorter course and do not belong in a cohort lagged by the full course length. Published cadre outputs regenerated to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TN_Health_Workforce_Projections_2050.xlsx
+++ b/TN_Health_Workforce_Projections_2050.xlsx
@@ -3539,7 +3539,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>0.9346380481340369</v>
+        <v>0.934792899408284</v>
       </c>
       <c r="E7" s="13" t="n">
         <v>0.8219931271477663</v>
@@ -3553,7 +3553,7 @@
         <v>10130</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>17935</v>
+        <v>17930</v>
       </c>
     </row>
     <row r="8">
@@ -4348,7 +4348,7 @@
         <v>392</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>8352</v>
+        <v>8350</v>
       </c>
       <c r="I4" s="8" t="n">
         <v>1558</v>
@@ -4418,7 +4418,7 @@
         <v>429</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>9275</v>
+        <v>9270</v>
       </c>
       <c r="I5" s="8" t="n">
         <v>1927</v>
@@ -4558,7 +4558,7 @@
         <v>452.799999999998</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>10910.49999999991</v>
+        <v>10909.99999999991</v>
       </c>
       <c r="I7" s="8" t="n">
         <v>2603.699999999962</v>
@@ -4628,7 +4628,7 @@
         <v>470.5999999999959</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>11690.99999999981</v>
+        <v>11689.99999999982</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>2898.399999999923</v>
@@ -4698,7 +4698,7 @@
         <v>488.3999999999938</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>12471.49999999972</v>
+        <v>12469.99999999972</v>
       </c>
       <c r="I9" s="8" t="n">
         <v>3193.099999999885</v>
@@ -4768,7 +4768,7 @@
         <v>506.1999999999917</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>13251.99999999963</v>
+        <v>13249.99999999963</v>
       </c>
       <c r="I10" s="8" t="n">
         <v>3487.799999999846</v>
@@ -4838,7 +4838,7 @@
         <v>523.9999999999897</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>14032.49999999954</v>
+        <v>14029.99999999954</v>
       </c>
       <c r="I11" s="8" t="n">
         <v>3782.499999999808</v>
@@ -4908,7 +4908,7 @@
         <v>541.7999999999877</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>14812.99999999945</v>
+        <v>14809.99999999945</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>4077.199999999769</v>
@@ -4978,7 +4978,7 @@
         <v>559.5999999999856</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>15593.49999999935</v>
+        <v>15589.99999999936</v>
       </c>
       <c r="I13" s="8" t="n">
         <v>4371.89999999973</v>
@@ -5048,7 +5048,7 @@
         <v>577.3999999999835</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>16373.99999999926</v>
+        <v>16369.99999999927</v>
       </c>
       <c r="I14" s="8" t="n">
         <v>4666.599999999693</v>
@@ -5118,7 +5118,7 @@
         <v>595.1999999999814</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>17154.49999999917</v>
+        <v>17149.99999999917</v>
       </c>
       <c r="I15" s="8" t="n">
         <v>4961.299999999654</v>
@@ -5188,7 +5188,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I16" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5258,7 +5258,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I17" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5328,7 +5328,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I18" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5398,7 +5398,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I19" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5468,7 +5468,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5538,7 +5538,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I21" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5608,7 +5608,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I22" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5678,7 +5678,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I23" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5748,7 +5748,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5818,7 +5818,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I25" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5888,7 +5888,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I26" s="8" t="n">
         <v>5255.999999999616</v>
@@ -5958,7 +5958,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I27" s="8" t="n">
         <v>5255.999999999616</v>
@@ -6028,7 +6028,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I28" s="8" t="n">
         <v>5255.999999999616</v>
@@ -6098,7 +6098,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>5255.999999999616</v>
@@ -6168,7 +6168,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I30" s="8" t="n">
         <v>5255.999999999616</v>
@@ -6238,7 +6238,7 @@
         <v>612.9999999999794</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>17934.99999999908</v>
+        <v>17929.99999999908</v>
       </c>
       <c r="I31" s="8" t="n">
         <v>5255.999999999616</v>

</xml_diff>

<commit_message>
Population grows after 2025; WHO requirement rises with it; population on every chart
Published default is now the NCP series verbatim to 2025, then its own
2021 to 2025 rate (0.298 per cent a year) held constant. 2050 population
83.3 million, WHO requirement 92,659, density 62.2 per 10,000. The NCP
plateau remains as a sidebar option (68.1 per 10,000). Active doctors
are unchanged at 517,657 because supply does not depend on population.

Workbook, CSVs, model and provenance regenerated; Inputs B28 is a live
formula for the growth rate; dashboard engine verified at 0.000000
against the model on every series.

Charts: population in millions on a right-hand axis, one colour
throughout, with a sidebar toggle. Legends no longer overlap (chart
font measured from an installed face) and hover boxes are never clipped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TN_Health_Workforce_Projections_2050.xlsx
+++ b/TN_Health_Workforce_Projections_2050.xlsx
@@ -2762,7 +2762,7 @@
         <v>557686</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>73.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
     </row>
@@ -2780,7 +2780,7 @@
         <v>517657</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>68.09999999999999</v>
+        <v>62.2</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         <v>469842</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>61.8</v>
+        <v>56.4</v>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
     </row>
@@ -2820,7 +2820,7 @@
         <v>417894</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>55</v>
+        <v>50.2</v>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
     </row>
@@ -11732,17 +11732,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2011-2036: official NCP values used verbatim. 2037-2050: Pop(t) = Pop(t-1) x (1 + g(t)), where g falls linearly from -0.0038%/yr in 2036 to -0.35%/yr in 2050.</t>
+          <t>2011-2025: official NCP values used verbatim. 2026-2050: Pop(t) = Pop(t-1) x (1 + g), where g is the NCP series' own 2021 to 2025 average annual rate, 0.298 per cent, held constant (Inputs B28).</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>NCP published table, 26 annual values</t>
+          <t>NCP published table, 15 annual values to 2025</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019). Extension beyond 2036 is our own; TFR from SRS. Code: lines 49-68</t>
+          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019). The NCP series itself plateaus near 78 million from 2031; holding its recent rate instead is our choice so that the WHO requirement keeps rising with the population. Code: build_population()</t>
         </is>
       </c>
     </row>
@@ -12247,22 +12247,22 @@
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Population growth beyond 2036, falling to -0.35 per cent by 2050</t>
+          <t>Population growth beyond 2025, 0.30 per cent a year held constant</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>OWN ASSUMPTION</t>
+          <t>OWN CHOICE, RATE FROM NCP</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>The official NCP series stops at 2036 and its tail is a flat -3,000 per year stub, so it is not extended mechanically. The growth rate is instead taken to decline linearly to -0.35 per cent by 2050, reflecting demographic momentum exhausting at a TFR near 1.4.</t>
+          <t>The NCP series is used verbatim to 2025. Its 2021 to 2025 average rate is then held constant to 2050, so the population reaches 83.3 million and the WHO requirement rises with it. The NCP series itself plateaus near 78 million from 2031; that path gives 76.0 million in 2050 and is kept as an alternative in the dashboard.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Low impact. Moves the density denominator by under 2 per cent.</t>
+          <t>Moderate. Density in 2050 is 62.2 per 10,000 on this path against 68.1 on the NCP plateau; the surplus finding holds on both.</t>
         </is>
       </c>
     </row>
@@ -12544,17 +12544,17 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>NCP projection 2011-2036</t>
+          <t>NCP projection 2011-2025</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>72.1M to 78.07M</t>
+          <t>72.1M to 77.3M</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019).</t>
+          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019). Used verbatim to 2025.</t>
         </is>
       </c>
     </row>
@@ -12566,17 +12566,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Growth rate beyond 2036</t>
+          <t>Growth rate beyond 2025</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>declines linearly to -0.35%/yr by 2050</t>
+          <t>0.298%/yr, held constant to 2050</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Own extension. Tamil Nadu TFR approximately 1.3 to 1.4 (SRS), well below replacement. The NCP tail is itself a flat -3,000/yr linear stub, so it is not extended mechanically. Moves the density denominator by under 2%.</t>
+          <t>The NCP series' own 2021 to 2025 rate. Gives 83.3M in 2050. The NCP plateau (76.0M in 2050) is the alternative path in the dashboard.</t>
         </is>
       </c>
     </row>
@@ -13128,7 +13128,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>NCP / MoHFW official projections to 2036. Beyond 2036 the growth rate declines linearly to -0.35% per year by 2050, reflecting demographic momentum exhausting at a TFR near 1.4. Result: 77.32 million in 2025, peaking at 78.08 million in 2031, falling to 76.02 million by 2050.</t>
+          <t>NCP / MoHFW official projections used verbatim to 2025. From 2026 the population grows at the NCP series' own 2021 to 2025 rate, 0.298% per year, held constant. Result: 77.32 million in 2025, 79.89 million in 2036, 83.29 million in 2050. The NCP plateau near 78 million is kept as an alternative path in the dashboard.</t>
         </is>
       </c>
     </row>
@@ -13344,7 +13344,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Population beyond 2036 is our own extension, not an official projection. The model is state-level only, with no district, urban-rural, or public-private employment split. Superspecialty (DM and M.Ch) and DNB are folded into the PG account, since only one year of seat data exists for each.</t>
+          <t>Population beyond 2025 is our own extension, not an official projection. The model is state-level only, with no district, urban-rural, or public-private employment split. Superspecialty (DM and M.Ch) and DNB are folded into the PG account, since only one year of seat data exists for each.</t>
         </is>
       </c>
     </row>
@@ -14031,22 +14031,22 @@
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>ASSUMED BY US, NO SOURCE</t>
+          <t>ASSUMED BY US, RATE FROM SOURCE</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Population growth beyond 2036</t>
+          <t>Population growth beyond 2025</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Falling to minus 0.35 per cent by 2050</t>
+          <t>0.298 per cent a year, held constant</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Our own extension. The official series stops at 2036</t>
+          <t>The NCP series' 2021 to 2025 rate. The series itself plateaus from 2031</t>
         </is>
       </c>
     </row>
@@ -14102,17 +14102,17 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Population 2011 to 2036</t>
+          <t>Population 2011 to 2025</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>72.1M to 78.07M</t>
+          <t>72.1M to 77.3M</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population and MoHFW, Population Projections for India and States 2011-2036 (2019). Used verbatim, all 26 values</t>
+          <t>National Commission on Population and MoHFW, Population Projections for India and States 2011-2036 (2019). Used verbatim to 2025, 15 values</t>
         </is>
       </c>
     </row>
@@ -14178,7 +14178,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Sample Registration System. Used only to justify the population extension</t>
+          <t>Sample Registration System. Context for the NCP plateau; not used in the model</t>
         </is>
       </c>
     </row>
@@ -15852,7 +15852,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>DERIVED, see formula in cell B12: gap x fill x completion</t>
+          <t>DERIVED, see formula in cell B13: gap x fill x completion</t>
         </is>
       </c>
     </row>
@@ -16139,11 +16139,12 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Population growth rate at 2036</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="n">
-        <v>-3.842705264506212e-05</v>
+          <t>Population growth rate beyond 2025</t>
+        </is>
+      </c>
+      <c r="B28" s="9">
+        <f>(Projection!C16/Projection!C12)^(1/4)-1</f>
+        <v/>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -16152,27 +16153,27 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Implied by the NCP series tail</t>
+          <t>DERIVED, see formula in cell B28: NCP 2021 to 2025 average annual rate, held constant from 2026. The NCP series itself plateaus from 2031</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Population growth rate at 2050</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="n">
-        <v>-0.0035</v>
+          <t>Population, last NCP year used verbatim</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>2025</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>per year</t>
+          <t>year</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>OWN ASSUMPTION. Momentum exhausting at TFR near 1.4</t>
+          <t>The model's last observed year. NCP tail growth for reference: -0.0038% per year at 2036</t>
         </is>
       </c>
     </row>
@@ -17498,8 +17499,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
-        <v>77546000</v>
+      <c r="C17" s="8">
+        <f>C16*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D17" s="8">
         <f>IF(A17&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A17-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -17587,8 +17589,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>77653000</v>
+      <c r="C18" s="8">
+        <f>C17*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D18" s="8">
         <f>IF(A18&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A18-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -17676,8 +17679,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
-        <v>77761000</v>
+      <c r="C19" s="8">
+        <f>C18*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D19" s="8">
         <f>IF(A19&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A19-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -17765,8 +17769,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>77868000</v>
+      <c r="C20" s="8">
+        <f>C19*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D20" s="8">
         <f>IF(A20&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A20-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -17854,8 +17859,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
-        <v>77975000</v>
+      <c r="C21" s="8">
+        <f>C20*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D21" s="8">
         <f>IF(A21&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A21-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -17943,8 +17949,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>78082000</v>
+      <c r="C22" s="8">
+        <f>C21*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D22" s="8">
         <f>IF(A22&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A22-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18032,8 +18039,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
-        <v>78079000</v>
+      <c r="C23" s="8">
+        <f>C22*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D23" s="8">
         <f>IF(A23&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A23-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18121,8 +18129,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
-        <v>78076000</v>
+      <c r="C24" s="8">
+        <f>C23*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D24" s="8">
         <f>IF(A24&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A24-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18210,8 +18219,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n">
-        <v>78073000</v>
+      <c r="C25" s="8">
+        <f>C24*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D25" s="8">
         <f>IF(A25&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A25-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18299,8 +18309,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
-        <v>78070000</v>
+      <c r="C26" s="8">
+        <f>C25*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D26" s="8">
         <f>IF(A26&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A26-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18388,8 +18399,9 @@
           <t>Projected</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
-        <v>78067000</v>
+      <c r="C27" s="8">
+        <f>C26*(1+Inputs!$B$28)</f>
+        <v/>
       </c>
       <c r="D27" s="8">
         <f>IF(A27&gt;=Inputs!$B$23,Inputs!$B$22,ROUND((Inputs!$B$21+(Inputs!$B$22-Inputs!$B$21)*(A27-2025)/(Inputs!$B$23-2025))/50,0)*50)</f>
@@ -18478,7 +18490,7 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>C27*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A28-2036)/14))</f>
+        <f>C27*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D28" s="8">
@@ -18568,7 +18580,7 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>C28*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A29-2036)/14))</f>
+        <f>C28*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D29" s="8">
@@ -18658,7 +18670,7 @@
         </is>
       </c>
       <c r="C30" s="8">
-        <f>C29*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A30-2036)/14))</f>
+        <f>C29*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D30" s="8">
@@ -18748,7 +18760,7 @@
         </is>
       </c>
       <c r="C31" s="8">
-        <f>C30*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A31-2036)/14))</f>
+        <f>C30*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D31" s="8">
@@ -18838,7 +18850,7 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>C31*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A32-2036)/14))</f>
+        <f>C31*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D32" s="8">
@@ -18928,7 +18940,7 @@
         </is>
       </c>
       <c r="C33" s="8">
-        <f>C32*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A33-2036)/14))</f>
+        <f>C32*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D33" s="8">
@@ -19018,7 +19030,7 @@
         </is>
       </c>
       <c r="C34" s="8">
-        <f>C33*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A34-2036)/14))</f>
+        <f>C33*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D34" s="8">
@@ -19108,7 +19120,7 @@
         </is>
       </c>
       <c r="C35" s="8">
-        <f>C34*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A35-2036)/14))</f>
+        <f>C34*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D35" s="8">
@@ -19198,7 +19210,7 @@
         </is>
       </c>
       <c r="C36" s="8">
-        <f>C35*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A36-2036)/14))</f>
+        <f>C35*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D36" s="8">
@@ -19288,7 +19300,7 @@
         </is>
       </c>
       <c r="C37" s="8">
-        <f>C36*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A37-2036)/14))</f>
+        <f>C36*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D37" s="8">
@@ -19378,7 +19390,7 @@
         </is>
       </c>
       <c r="C38" s="8">
-        <f>C37*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A38-2036)/14))</f>
+        <f>C37*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D38" s="8">
@@ -19468,7 +19480,7 @@
         </is>
       </c>
       <c r="C39" s="8">
-        <f>C38*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A39-2036)/14))</f>
+        <f>C38*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D39" s="8">
@@ -19558,7 +19570,7 @@
         </is>
       </c>
       <c r="C40" s="8">
-        <f>C39*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A40-2036)/14))</f>
+        <f>C39*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D40" s="8">
@@ -19648,7 +19660,7 @@
         </is>
       </c>
       <c r="C41" s="8">
-        <f>C40*(1+(Inputs!$B$28+(Inputs!$B$29-Inputs!$B$28)*(A41-2036)/14))</f>
+        <f>C40*(1+Inputs!$B$28)</f>
         <v/>
       </c>
       <c r="D41" s="8">
@@ -19739,7 +19751,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Typed numbers appear only where a formula is not possible: published population (column C to 2036), observed seats and registrations to 2025,</t>
+          <t>Typed numbers appear only where a formula is not possible: published population (column C to 2025), observed seats and registrations to 2025,</t>
         </is>
       </c>
     </row>
@@ -19971,13 +19983,13 @@
         <v>19.6</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>45.2</v>
+        <v>43.5</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>64.2</v>
+        <v>58.6</v>
       </c>
     </row>
     <row r="9">
@@ -20163,13 +20175,13 @@
         <v>19.6</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46.3</v>
+        <v>44.6</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>68.09999999999999</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="17">
@@ -20355,13 +20367,13 @@
         <v>19.6</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>47.4</v>
+        <v>45.6</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>73.3</v>
+        <v>66.90000000000001</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
World Bank demand line, with full citations throughout
A rising benchmark from the same framework as the WHO floor: the demand
model of Liu, Goryakin, Maeda, Bruckner and Scheffler (2017, Table 1),
anchored on the modelled 2025 density and moved by GSDP per capita
(elasticity 0.244), out-of-pocket spending (-0.099) and the population
aged 65+ (0.516). Driver paths are assumptions marked for State
confirmation and editable in the sidebar. Demand reaches 305,668 by
2050 against supply of 517,657.

Model, engine (verified 0.000000), workbook (Inputs B32 to B38, live
columns X and Y), results and provenance documents, README and dashboard
all carry it. Full references written once and used wherever a source is
named: Liu et al. 2017, WHO 2016, WHO 2021, NCP 2019.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TN_Health_Workforce_Projections_2050.xlsx
+++ b/TN_Health_Workforce_Projections_2050.xlsx
@@ -11628,7 +11628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11742,7 +11742,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019). The NCP series itself plateaus near 78 million from 2031; holding its recent rate instead is our choice so that the WHO requirement keeps rising with the population. Code: build_population()</t>
+          <t>National Commission on Population, Ministry of Health and Family Welfare. Population Projections for India and States 2011-2036: Report of the Technical Group on Population Projections. New Delhi: Government of India; July 2019. The NCP series itself plateaus near 78 million from 2031; holding its recent rate instead is our choice so that the WHO requirement keeps rising with the population. Code: build_population()</t>
         </is>
       </c>
     </row>
@@ -12039,7 +12039,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>WHO, Global Strategy on Human Resources for Health: Workforce 2030 (2016) for 44.5; WHO (2016) for the 1:3 split. Code: lines 394-396</t>
+          <t>World Health Organization. Global Strategy on Human Resources for Health: Workforce 2030. Geneva: WHO; 2016. for 44.5; the same source for the 1:3 doctor to nurse split. Code: NEED_DOCTORS</t>
         </is>
       </c>
     </row>
@@ -12065,6 +12065,60 @@
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="92" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>World Bank demand (doctors)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>The number of doctors the economy would absorb, on the World Bank health labour market demand model. Rises with income, ageing and the shift away from out-of-pocket payment. A demand line, not a norm.</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ln(physicians per 1,000) = -9.882 + 0.231 ln GDPpc(t-1) + 0.531 ln GDPpc(t-4) - 0.518 ln GDPpc(t-5) - 0.099 ln OOPpc(t-2) + 0.516 ln Pop65(t-3) + country effect (Table 1). The country effect pins the level, so the series is anchored on the modelled 2025 density and moved each year by the three drivers: density(t) = density(t-1) x (1+g)^0.244 x (1+g+adj)^-0.099 x (1+p65)^0.516, times population. Inputs B32 to B38.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Published elasticities; three assumed growth paths (Inputs B35 to B38)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. Code: build_wb_demand()</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="92" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Surplus vs WB demand</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>How far supply runs above what the economy would absorb.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Active doctors - World Bank demand.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
@@ -12081,7 +12135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12247,64 +12301,86 @@
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Population growth beyond 2025, 0.30 per cent a year held constant</t>
+          <t>World Bank demand line: growth paths of its three drivers</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>OWN CHOICE, RATE FROM NCP</t>
+          <t>ASSUMED, FOR STATE CONFIRMATION</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>The NCP series is used verbatim to 2025. Its 2021 to 2025 average rate is then held constant to 2050, so the population reaches 83.3 million and the WHO requirement rises with it. The NCP series itself plateaus near 78 million from 2031; that path gives 76.0 million in 2050 and is kept as an alternative in the dashboard.</t>
+          <t>The elasticities are published (Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016., Table 1): 0.244 to real GDP per capita in the long run, -0.099 to out-of-pocket spending per capita, 0.516 to the population aged 65 and over. What is assumed is the path of the drivers: real GSDP per capita growth of 6.5 per cent in 2026 easing to 4.0 per cent by 2050, out-of-pocket spending growing with GDP (share constant), and the 65+ population growing 3.5 per cent a year. The State's own GSDP forecast and the NCP 2019 age tables should replace these. The line is anchored on the modelled 2025 density, which is how the paper's country fixed effect works.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Moderate. Density in 2050 is 62.2 per 10,000 on this path against 68.1 on the NCP plateau; the surplus finding holds on both.</t>
+          <t>Moderate. Demand reaches 305,668 by 2050 on these paths; supply is 517,657. A faster economy raises the line, but with an elasticity of 0.244 it would take implausible growth to close the gap.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="128" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Completion rate, 95 per cent for medical courses</t>
+          <t>Population growth beyond 2025, 0.30 per cent a year held constant</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>BENCHMARK, validated</t>
+          <t>OWN CHOICE, RATE FROM NCP</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Taken as the NMC benchmark and also used in the Andhra Pradesh model. It is not estimated from Tamil Nadu data directly for MBBS because no admission cohort in the observed window can be matched to its own pass-out year at a 6-year lag. It was validated indirectly on PG, where the match is possible: predicted 2,707 against 2,717 observed.</t>
+          <t>The NCP series is used verbatim to 2025. Its 2021 to 2025 average rate is then held constant to 2050, so the population reaches 83.3 million and the WHO requirement rises with it. The NCP series itself plateaus near 78 million from 2031; that path gives 76.0 million in 2050 and is kept as an alternative in the dashboard.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>None outstanding.</t>
+          <t>Moderate. Density in 2050 is 62.2 per 10,000 on this path against 68.1 on the NCP plateau; the surplus finding holds on both.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="128" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>Completion rate, 95 per cent for medical courses</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>BENCHMARK, validated</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Taken as the NMC benchmark and also used in the Andhra Pradesh model. It is not estimated from Tamil Nadu data directly for MBBS because no admission cohort in the observed window can be matched to its own pass-out year at a 6-year lag. It was validated indirectly on PG, where the match is possible: predicted 2,707 against 2,717 observed.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>None outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="128" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Cadre seat growth: frozen, or trend continued to 2035 then held</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>OWN ASSUMPTION</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>With four or five annual observations per cadre a fitted ceiling cannot be supported, so two bounding paths are given instead. Holding flat after 2035 reflects that capacity cannot expand indefinitely against a falling state population.</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>FOR STATE CONFIRMATION alongside the medical seat paths.</t>
         </is>
@@ -12554,7 +12630,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population / MoHFW, Population Projections for India and States 2011-2036 (2019). Used verbatim to 2025.</t>
+          <t>National Commission on Population, Ministry of Health and Family Welfare. Population Projections for India and States 2011-2036: Report of the Technical Group on Population Projections. New Delhi: Government of India; July 2019. Used verbatim to 2025.</t>
         </is>
       </c>
     </row>
@@ -13053,7 +13129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13080,7 +13156,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>A stock-and-flow supply model with an explicit education pipeline, following the WHO / World Bank Health Labour Market Framework as operationalised in Liu, Goryakin, Maeda, Bruckner and Scheffler, Global Health Workforce Labor Market Projections for 2030 (World Bank Policy Research Working Paper 7790; Human Resources for Health 2017;15:11), and in the WHO Health Labour Market Analysis Guidebook (2021). The same three-lens structure, Supply, Need and Demand, used in the Centre's Andhra Pradesh projection. This round builds the Supply lens for Tamil Nadu and extends the horizon to 2050.</t>
+          <t>A stock-and-flow supply model with an explicit education pipeline, following the WHO / World Bank Health Labour Market Framework as operationalised in Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. and in World Health Organization. Health Labour Market Analysis Guidebook. Geneva: WHO; 2021. The same three-lens structure, Supply, Need and Demand, used in the Centre's Andhra Pradesh projection. This round builds the Supply lens for Tamil Nadu to 2050, sets it against the WHO need floor, and adds the World Bank demand line from the same paper.</t>
         </is>
       </c>
     </row>
@@ -13135,214 +13211,226 @@
     <row r="7" ht="74" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Module 2, seats</t>
+          <t>Module 6b, demand benchmark</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Government and private modelled separately because they are on different trajectories. Government is a step and scenario process. Private follows bounded logistic growth fitted in levels at three ceilings. PG seats grow linearly, capped at 70% of total MBBS seats.</t>
+          <t>Doctors the economy would absorb, on the demand model of Liu et al. 2017: ln(physicians per 1,000) = -9.882 + 0.231 ln GDPpc(t-1) + 0.531 ln GDPpc(t-4) - 0.518 ln GDPpc(t-5) - 0.099 ln OOPpc(t-2) + 0.516 ln Pop65(t-3) + country effect, estimated by GLM with country fixed effects on 165 countries, 1990 to 2013. The country effect pins the level, so the line is anchored on Tamil Nadu's modelled 2025 density and moved by the three drivers, whose growth paths are assumptions marked for State confirmation. Result: 151,248 in 2025, 233,187 in 2040, 305,668 in 2050. Supply exceeds it throughout; the gap is 211,989 doctors in 2050.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="74" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Module 3, pipeline</t>
+          <t>Module 2, seats</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Seats to admissions via the fill rate, admissions to graduates via the completion rate, graduates to the register with a lag. Fill rates are estimated directly from MGRMU sanctioned-against-admitted data: 99.8% for MBBS, 97.8% for PG. Completion is 95%. The MBBS lag is six years, being 4.5 academic years plus a twelve-month internship; the PG lag is three years.</t>
+          <t>Government and private modelled separately because they are on different trajectories. Government is a step and scenario process. Private follows bounded logistic growth fitted in levels at three ceilings. PG seats grow linearly, capped at 70% of total MBBS seats.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="74" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Module 4, external entrants</t>
+          <t>Module 3, pipeline</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The residual between observed registrations and modelled domestic output, decomposed into foreign medical graduates, which are observed and projected linearly to a ceiling of 3,000, and deemed-university plus out-of-state entrants, held flat at the observed mean because the five observations show no trend.</t>
+          <t>Seats to admissions via the fill rate, admissions to graduates via the completion rate, graduates to the register with a lag. Fill rates are estimated directly from MGRMU sanctioned-against-admitted data: 99.8% for MBBS, 97.8% for PG. Completion is 95%. The MBBS lag is six years, being 4.5 academic years plus a twelve-month internship; the PG lag is three years.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="74" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Module 5, stock and flow</t>
+          <t>Module 4, external entrants</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Register cohorts are rolled forward from 1927, with age inferred from registration year at an assumed age of 24. Three separate outflows apply: age-specific mortality; emigration and out-of-state loss at 1.2% per year across ages 25 to 45; and a retirement hazard reducing participation from age 60.</t>
+          <t>The residual between observed registrations and modelled domestic output, decomposed into foreign medical graduates, which are observed and projected linearly to a ceiling of 3,000, and deemed-university plus out-of-state entrants, held flat at the observed mean because the five observations show no trend.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="74" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Module 6, specialists</t>
+          <t>Module 5, stock and flow</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Specialists are tracked as a transition within the stock, never as an addition to it. An MD or MS entrant is an already-registered MBBS doctor, so adding PG output to MBBS output would double-count every specialist.</t>
+          <t>Register cohorts are rolled forward from 1927, with age inferred from registration year at an assumed age of 24. Three separate outflows apply: age-specific mortality; emigration and out-of-state loss at 1.2% per year across ages 25 to 45; and a retirement hazard reducing participation from age 60.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="74" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Deemed overlap correction</t>
+          <t>Module 6, specialists</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>The Selection Committee and MGRMU private MBBS seat series agree exactly for 2021-22 and 2022-23, then diverge by 450, 550 and 850 seats. The gap is most likely deemed universities entering the Committee sheet. Because deemed output is already inside the external-entrant residual, which was estimated from years when the two sources agreed, those graduates would otherwise be counted twice. The correction is 850 x 0.998 x 0.95 = 806 graduates per year, applied from registration year 2031, with the smaller observed gaps used for 2029 and 2030.</t>
+          <t>Specialists are tracked as a transition within the stock, never as an addition to it. An MD or MS entrant is an already-registered MBBS doctor, so adding PG output to MBBS output would double-count every specialist.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="74" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Live formulas</t>
+          <t>Deemed overlap correction</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>The workbook computes rather than reports. Every parameter sits in one cell on the Inputs sheet and the model sheets reference it, so a reviewer can change an assumption and watch the projection move. Typed numbers appear only where a formula is not possible: published population data, observed seats and registrations, and the three cohort-model flows (retirements, deaths, migration) which depend on the full age distribution of the register. Every formula column was checked cell by cell against the model and reproduces it exactly.</t>
+          <t>The Selection Committee and MGRMU private MBBS seat series agree exactly for 2021-22 and 2022-23, then diverge by 450, 550 and 850 seats. The gap is most likely deemed universities entering the Committee sheet. Because deemed output is already inside the external-entrant residual, which was estimated from years when the two sources agreed, those graduates would otherwise be counted twice. The correction is 850 x 0.998 x 0.95 = 806 graduates per year, applied from registration year 2031, with the smaller observed gaps used for 2029 and 2030.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="74" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Live formulas</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>The model was tested against data it was not fitted to. The scraped register and the TNMC workbook agree to within 0.17%, and exactly in 2024. The PG pipeline predicted 2,707 pass-outs for 2024 against 2,717 observed. The PG coverage factor gives 4,630 against an independent 4,629.</t>
+          <t>The workbook computes rather than reports. Every parameter sits in one cell on the Inputs sheet and the model sheets reference it, so a reviewer can change an assumption and watch the projection move. Typed numbers appear only where a formula is not possible: published population data, observed seats and registrations, and the three cohort-model flows (retirements, deaths, migration) which depend on the full age distribution of the register. Every formula column was checked cell by cell against the model and reproduces it exactly.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="74" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Key caveat</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>This is an unconstrained supply projection. It answers how many doctors Tamil Nadu will produce and retain on current trajectories, not how many the health system will employ. A 2050 density of 68.7 per 10,000, about twice the OECD average, is the model reporting that current seat-expansion trajectories exceed any plausible absorption capacity. That is the finding, not a forecast of employment.</t>
+          <t>The model was tested against data it was not fitted to. The scraped register and the TNMC workbook agree to within 0.17%, and exactly in 2024. The PG pipeline predicted 2,707 pass-outs for 2024 against 2,717 observed. The PG coverage factor gives 4,630 against an independent 4,629.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="74" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Limitation, seat sources</t>
+          <t>Key caveat</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>The Selection Committee and MGRMU disagree on private MBBS seats from 2023, being 4,750 against 3,900 in 2025-26. The gap is most likely deemed universities. The model uses the Selection Committee basis and places deemed output in the external residual.</t>
+          <t>This is an unconstrained supply projection. It answers how many doctors Tamil Nadu will produce and retain on current trajectories, not how many the health system will employ. A 2050 density of 68.7 per 10,000, about twice the OECD average, is the model reporting that current seat-expansion trajectories exceed any plausible absorption capacity. That is the finding, not a forecast of employment.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="74" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Limitation, emigration</t>
+          <t>Limitation, seat sources</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>The emigration parameter is calibrated, not observed. No direct measure of Tamil Nadu doctor out-migration exists. The Sensitivity sheet prices the uncertainty.</t>
+          <t>The Selection Committee and MGRMU disagree on private MBBS seats from 2023, being 4,750 against 3,900 in 2025-26. The gap is most likely deemed universities. The model uses the Selection Committee basis and places deemed output in the external residual.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="74" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Limitation, age</t>
+          <t>Limitation, emigration</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Age is inferred from registration year, not observed. Retirement timing is the figure most sensitive to this assumption.</t>
+          <t>The emigration parameter is calibrated, not observed. No direct measure of Tamil Nadu doctor out-migration exists. The Sensitivity sheet prices the uncertainty.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="74" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Other cadres, scope</t>
+          <t>Limitation, age</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Nursing at degree level, dental, pharmacy, physiotherapy and occupational therapy, the five AYUSH streams and allied health at postgraduate level are projected on the same chain as doctors: seats, fill rate, completion rate, course length lag. Twenty cadres in all. Every rate is estimated from the MGRMU files rather than assumed, except where the Cadre parameters sheet records it as assumed.</t>
+          <t>Age is inferred from registration year, not observed. Retirement timing is the figure most sensitive to this assumption.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="74" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Other cadres, what these figures are NOT</t>
+          <t>Other cadres, scope</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>These are annual qualified output, not a practising workforce. No register comparable to the National Medical Commission register exists for any of these cadres, so there is no opening stock, no attrition for death, retirement or migration, and no need or demand benchmark. They cannot be added to the doctor stock, and a practising total across all cadres is not possible from this data.</t>
+          <t>Nursing at degree level, dental, pharmacy, physiotherapy and occupational therapy, the five AYUSH streams and allied health at postgraduate level are projected on the same chain as doctors: seats, fill rate, completion rate, course length lag. Twenty cadres in all. Every rate is estimated from the MGRMU files rather than assumed, except where the Cadre parameters sheet records it as assumed.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="74" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Other cadres, fill rates</t>
+          <t>Other cadres, what these figures are NOT</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Fill rates outside medicine are far lower and matter far more. MBBS runs at 99 per cent of sanctioned seats filled, but Post Basic BSc Nursing is at 48 per cent, MSc Nursing 59, allied health PG 65 and BHMS 66. For those cadres sanctioned seats overstate real output substantially, which is why the model runs on admissions.</t>
+          <t>These are annual qualified output, not a practising workforce. No register comparable to the National Medical Commission register exists for any of these cadres, so there is no opening stock, no attrition for death, retirement or migration, and no need or demand benchmark. They cannot be added to the doctor stock, and a practising total across all cadres is not possible from this data.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="74" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Other cadres, seat growth</t>
+          <t>Other cadres, fill rates</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>With four or five annual observations per cadre a fitted ceiling cannot be supported, so two paths are given: seats frozen at the last observed level, and the fitted linear trend continued to 2035 then held flat. Fitted in levels, never as a compound rate. Totals begin at 2027, the first year in which every course length has a source cohort, since seat data starts in 2021 and the longest course is six years.</t>
+          <t>Fill rates outside medicine are far lower and matter far more. MBBS runs at 99 per cent of sanctioned seats filled, but Post Basic BSc Nursing is at 48 per cent, MSc Nursing 59, allied health PG 65 and BHMS 66. For those cadres sanctioned seats overstate real output substantially, which is why the model runs on admissions.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="74" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Other cadres, known gaps</t>
+          <t>Other cadres, seat growth</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>GNM and ANM nursing are absent from every source file because they sit with the Tamil Nadu Nurses and Midwives Council rather than the university, so nursing here is degree level only and understates total nursing output. Allied health at degree level is present but internally inconsistent and is excluded. Twelve single pass-out years across various cadres were excluded as partial extracts. All of this is itemised on the Data quality and Not covered sheets.</t>
+          <t>With four or five annual observations per cadre a fitted ceiling cannot be supported, so two paths are given: seats frozen at the last observed level, and the fitted linear trend continued to 2035 then held flat. Fitted in levels, never as a compound rate. Totals begin at 2027, the first year in which every course length has a source cohort, since seat data starts in 2021 and the longest course is six years.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="74" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>Other cadres, known gaps</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>GNM and ANM nursing are absent from every source file because they sit with the Tamil Nadu Nurses and Midwives Council rather than the university, so nursing here is degree level only and understates total nursing output. Allied health at degree level is present but internally inconsistent and is excluded. Twelve single pass-out years across various cadres were excluded as partial extracts. All of this is itemised on the Data quality and Not covered sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="74" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>Limitation, other</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Population beyond 2025 is our own extension, not an official projection. The model is state-level only, with no district, urban-rural, or public-private employment split. Superspecialty (DM and M.Ch) and DNB are folded into the PG account, since only one year of seat data exists for each.</t>
         </is>
@@ -13359,7 +13447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14112,7 +14200,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>National Commission on Population and MoHFW, Population Projections for India and States 2011-2036 (2019). Used verbatim to 2025, 15 values</t>
+          <t>National Commission on Population, Ministry of Health and Family Welfare. Population Projections for India and States 2011-2036: Report of the Technical Group on Population Projections. New Delhi: Government of India; July 2019. Used verbatim to 2025, 15 values</t>
         </is>
       </c>
     </row>
@@ -14124,39 +14212,39 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WHO density norm</t>
+          <t>World Bank demand elasticities</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>44.5 per 10,000</t>
+          <t>0.244 income, -0.099 out-of-pocket, 0.516 population 65+</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>WHO, Global Strategy on HRH: Workforce 2030 (2016)</t>
+          <t>Table 1 of Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="40" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>EXTERNAL PUBLISHED SOURCE</t>
+          <t>ASSUMED BY US, FOR STATE CONFIRMATION</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Doctor share of the norm</t>
+          <t>World Bank demand driver paths</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>One quarter</t>
+          <t>GSDP per capita 6.5% easing to 4.0%; OOP share constant; 65+ population 3.5%/yr</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>WHO (2016), doctor to nurse 1 to 3</t>
+          <t>Our own. To be replaced by the State's GSDP forecast and the NCP 2019 age tables</t>
         </is>
       </c>
     </row>
@@ -14168,17 +14256,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Total fertility rate</t>
+          <t>WHO density norm</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>About 1.3 to 1.4</t>
+          <t>44.5 per 10,000</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Sample Registration System. Context for the NCP plateau; not used in the model</t>
+          <t>WHO, Global Strategy on HRH: Workforce 2030 (2016)</t>
         </is>
       </c>
     </row>
@@ -14190,66 +14278,110 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>NMC seat ceiling per college</t>
+          <t>Doctor share of the norm</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>250 MBBS seats</t>
+          <t>One quarter</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>National Medical Commission norms</t>
+          <t>WHO (2016), doctor to nurse 1 to 3</t>
         </is>
       </c>
     </row>
     <row r="39" ht="40" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>EXTERNAL PUBLISHED SOURCE</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Total fertility rate</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>About 1.3 to 1.4</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Sample Registration System. Context for the NCP plateau; not used in the model</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>EXTERNAL PUBLISHED SOURCE</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>NMC seat ceiling per college</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>250 MBBS seats</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>National Medical Commission norms</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
           <t>SCRAPED BY US</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Full TNMC register</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>193,264 doctors, 1927 to 2025</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>NMC Indian Medical Register, scraped via run_all.py, endpoint nmc.org.in/MCIRest/open/getPaginatedData, state council id 21</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Roughly 60 per cent of the figures come straight from the supplied files or are computed from them. About 25 per cent are external published sources, almost all of that the population series and the WHO norm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>About 15 per cent are our own assumptions. Five of those matter: the private seat ceilings, the PG cap, the government seat targets, the emigration rate and age at registration.</t>
-        </is>
-      </c>
-    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>The first three need the State's confirmation. The last two need data that exists but we do not hold: the NMC detail records carry birth dates and removal status.</t>
+          <t>Roughly 60 per cent of the figures come straight from the supplied files or are computed from them. About 25 per cent are external published sources, almost all of that the population series and the WHO norm.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>About 15 per cent are our own assumptions. Five of those matter: the private seat ceilings, the PG cap, the government seat targets, the emigration rate and age at registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>The first three need the State's confirmation. The last two need data that exists but we do not hold: the NMC detail records carry birth dates and removal status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Data altered or excluded is on the Data quality sheet. Cadres not projected are on the Not covered sheet. Neither was dropped silently.</t>
         </is>
@@ -14787,7 +14919,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>https://nhm.gov.in/New_Updates_2018/Report_Population_Projection_2019.pdf</t>
+          <t>National Commission on Population, Ministry of Health and Family Welfare. Population Projections for India and States 2011-2036: Report of the Technical Group on Population Projections. New Delhi: Government of India; July 2019. https://nhm.gov.in/New_Updates_2018/Report_Population_Projection_2019.pdf</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -15105,7 +15237,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Liu, Goryakin, Maeda, Bruckner and Scheffler, World Bank</t>
+          <t>Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -15115,17 +15247,17 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>The principal method reference: the supply, need and demand framework</t>
+          <t>The principal method reference: the supply, need and demand framework, and the demand elasticities in Table 1 used for the World Bank demand line</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>World Bank Policy Research Working Paper 7790; Human Resources for Health 2017;15:11</t>
+          <t>Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. https://doi.org/10.1186/s12960-017-0187-2 ; working paper at https://documents1.worldbank.org/curated/en/546161470834083341/pdf/WPS7790.pdf</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Method reference</t>
+          <t>Verified, coefficients read from Table 1</t>
         </is>
       </c>
     </row>
@@ -15157,7 +15289,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>WHO, Geneva</t>
+          <t>World Health Organization. Health Labour Market Analysis Guidebook. Geneva: WHO; 2021. https://www.who.int/publications/i/item/9789240035546</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -15194,7 +15326,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>WHO, Geneva</t>
+          <t>World Health Organization. Global Strategy on Human Resources for Health: Workforce 2030. Geneva: WHO; 2016. https://www.who.int/publications/i/item/9789241511131</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -15584,7 +15716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -16214,6 +16346,146 @@
       <c r="D31" s="3" t="inlineStr">
         <is>
           <t>INFERRED, not observed. See Age sensitivity sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: income elasticity</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>elasticity</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>PUBLISHED. Sum of the three GDP per capita lags in Table 1, 0.231 + 0.531 - 0.518, of Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: out-of-pocket elasticity</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>-0.099</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>elasticity</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>PUBLISHED. Table 1 of Liu et al. 2017 (full reference in row 32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: population 65+ elasticity</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>elasticity</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>PUBLISHED. Table 1 of Liu et al. 2017 (full reference in row 32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: real GSDP per capita growth, 2026</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED, FOR STATE CONFIRMATION. Recent Tamil Nadu real GSDP growth less population growth. See Assumptions sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: real GSDP per capita growth, 2050</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED, FOR STATE CONFIRMATION. The 2026 rate eases linearly to this by 2050</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: OOP growth less GDP growth</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED. Zero holds the out-of-pocket share of spending constant</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>WB demand: growth of population aged 65+</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED, FOR STATE CONFIRMATION. To be replaced by the NCP 2019 age tables for Tamil Nadu</t>
         </is>
       </c>
     </row>
@@ -16228,7 +16500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W46"/>
+  <dimension ref="A1:Y46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16254,6 +16526,8 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -16370,6 +16644,16 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Surplus vs WHO need</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>World Bank demand (doctors)</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Surplus vs WB demand</t>
         </is>
       </c>
     </row>
@@ -16436,6 +16720,8 @@
         <f>Q2-V2</f>
         <v/>
       </c>
+      <c r="X2" s="8" t="n"/>
+      <c r="Y2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -16502,6 +16788,8 @@
         <f>Q3-V3</f>
         <v/>
       </c>
+      <c r="X3" s="8" t="n"/>
+      <c r="Y3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -16568,6 +16856,8 @@
         <f>Q4-V4</f>
         <v/>
       </c>
+      <c r="X4" s="8" t="n"/>
+      <c r="Y4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -16634,6 +16924,8 @@
         <f>Q5-V5</f>
         <v/>
       </c>
+      <c r="X5" s="8" t="n"/>
+      <c r="Y5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -16707,6 +16999,8 @@
         <f>Q6-V6</f>
         <v/>
       </c>
+      <c r="X6" s="8" t="n"/>
+      <c r="Y6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -16780,6 +17074,8 @@
         <f>Q7-V7</f>
         <v/>
       </c>
+      <c r="X7" s="8" t="n"/>
+      <c r="Y7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -16853,6 +17149,8 @@
         <f>Q8-V8</f>
         <v/>
       </c>
+      <c r="X8" s="8" t="n"/>
+      <c r="Y8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -16926,6 +17224,8 @@
         <f>Q9-V9</f>
         <v/>
       </c>
+      <c r="X9" s="8" t="n"/>
+      <c r="Y9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -16999,6 +17299,8 @@
         <f>Q10-V10</f>
         <v/>
       </c>
+      <c r="X10" s="8" t="n"/>
+      <c r="Y10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -17074,6 +17376,8 @@
         <f>Q11-V11</f>
         <v/>
       </c>
+      <c r="X11" s="8" t="n"/>
+      <c r="Y11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -17157,6 +17461,8 @@
         <f>Q12-V12</f>
         <v/>
       </c>
+      <c r="X12" s="8" t="n"/>
+      <c r="Y12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -17240,6 +17546,8 @@
         <f>Q13-V13</f>
         <v/>
       </c>
+      <c r="X13" s="8" t="n"/>
+      <c r="Y13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -17323,6 +17631,8 @@
         <f>Q14-V14</f>
         <v/>
       </c>
+      <c r="X14" s="8" t="n"/>
+      <c r="Y14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -17406,6 +17716,8 @@
         <f>Q15-V15</f>
         <v/>
       </c>
+      <c r="X15" s="8" t="n"/>
+      <c r="Y15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -17489,6 +17801,14 @@
         <f>Q16-V16</f>
         <v/>
       </c>
+      <c r="X16" s="8">
+        <f>Q16</f>
+        <v/>
+      </c>
+      <c r="Y16" s="8">
+        <f>Q16-X16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -17579,6 +17899,14 @@
         <f>Q17-V17</f>
         <v/>
       </c>
+      <c r="X17" s="8">
+        <f>X16/C16*C17*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A17-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A17-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y17" s="8">
+        <f>Q17-X17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -17669,6 +17997,14 @@
         <f>Q18-V18</f>
         <v/>
       </c>
+      <c r="X18" s="8">
+        <f>X17/C17*C18*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A18-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A18-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y18" s="8">
+        <f>Q18-X18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -17759,6 +18095,14 @@
         <f>Q19-V19</f>
         <v/>
       </c>
+      <c r="X19" s="8">
+        <f>X18/C18*C19*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A19-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A19-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y19" s="8">
+        <f>Q19-X19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -17849,6 +18193,14 @@
         <f>Q20-V20</f>
         <v/>
       </c>
+      <c r="X20" s="8">
+        <f>X19/C19*C20*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A20-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A20-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y20" s="8">
+        <f>Q20-X20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -17939,6 +18291,14 @@
         <f>Q21-V21</f>
         <v/>
       </c>
+      <c r="X21" s="8">
+        <f>X20/C20*C21*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A21-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A21-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y21" s="8">
+        <f>Q21-X21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -18029,6 +18389,14 @@
         <f>Q22-V22</f>
         <v/>
       </c>
+      <c r="X22" s="8">
+        <f>X21/C21*C22*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A22-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A22-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y22" s="8">
+        <f>Q22-X22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -18119,6 +18487,14 @@
         <f>Q23-V23</f>
         <v/>
       </c>
+      <c r="X23" s="8">
+        <f>X22/C22*C23*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A23-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A23-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y23" s="8">
+        <f>Q23-X23</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -18209,6 +18585,14 @@
         <f>Q24-V24</f>
         <v/>
       </c>
+      <c r="X24" s="8">
+        <f>X23/C23*C24*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A24-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A24-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y24" s="8">
+        <f>Q24-X24</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -18299,6 +18683,14 @@
         <f>Q25-V25</f>
         <v/>
       </c>
+      <c r="X25" s="8">
+        <f>X24/C24*C25*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A25-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A25-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y25" s="8">
+        <f>Q25-X25</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -18389,6 +18781,14 @@
         <f>Q26-V26</f>
         <v/>
       </c>
+      <c r="X26" s="8">
+        <f>X25/C25*C26*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A26-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A26-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y26" s="8">
+        <f>Q26-X26</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -18479,6 +18879,14 @@
         <f>Q27-V27</f>
         <v/>
       </c>
+      <c r="X27" s="8">
+        <f>X26/C26*C27*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A27-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A27-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y27" s="8">
+        <f>Q27-X27</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -18569,6 +18977,14 @@
         <f>Q28-V28</f>
         <v/>
       </c>
+      <c r="X28" s="8">
+        <f>X27/C27*C28*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A28-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A28-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y28" s="8">
+        <f>Q28-X28</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -18659,6 +19075,14 @@
         <f>Q29-V29</f>
         <v/>
       </c>
+      <c r="X29" s="8">
+        <f>X28/C28*C29*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A29-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A29-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y29" s="8">
+        <f>Q29-X29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -18749,6 +19173,14 @@
         <f>Q30-V30</f>
         <v/>
       </c>
+      <c r="X30" s="8">
+        <f>X29/C29*C30*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A30-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A30-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y30" s="8">
+        <f>Q30-X30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -18839,6 +19271,14 @@
         <f>Q31-V31</f>
         <v/>
       </c>
+      <c r="X31" s="8">
+        <f>X30/C30*C31*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A31-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A31-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y31" s="8">
+        <f>Q31-X31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -18929,6 +19369,14 @@
         <f>Q32-V32</f>
         <v/>
       </c>
+      <c r="X32" s="8">
+        <f>X31/C31*C32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A32-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A32-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y32" s="8">
+        <f>Q32-X32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -19019,6 +19467,14 @@
         <f>Q33-V33</f>
         <v/>
       </c>
+      <c r="X33" s="8">
+        <f>X32/C32*C33*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A33-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A33-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y33" s="8">
+        <f>Q33-X33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -19109,6 +19565,14 @@
         <f>Q34-V34</f>
         <v/>
       </c>
+      <c r="X34" s="8">
+        <f>X33/C33*C34*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A34-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A34-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y34" s="8">
+        <f>Q34-X34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -19199,6 +19663,14 @@
         <f>Q35-V35</f>
         <v/>
       </c>
+      <c r="X35" s="8">
+        <f>X34/C34*C35*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A35-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A35-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y35" s="8">
+        <f>Q35-X35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -19289,6 +19761,14 @@
         <f>Q36-V36</f>
         <v/>
       </c>
+      <c r="X36" s="8">
+        <f>X35/C35*C36*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A36-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A36-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y36" s="8">
+        <f>Q36-X36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -19379,6 +19859,14 @@
         <f>Q37-V37</f>
         <v/>
       </c>
+      <c r="X37" s="8">
+        <f>X36/C36*C37*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A37-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A37-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y37" s="8">
+        <f>Q37-X37</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -19469,6 +19957,14 @@
         <f>Q38-V38</f>
         <v/>
       </c>
+      <c r="X38" s="8">
+        <f>X37/C37*C38*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A38-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A38-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y38" s="8">
+        <f>Q38-X38</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -19559,6 +20055,14 @@
         <f>Q39-V39</f>
         <v/>
       </c>
+      <c r="X39" s="8">
+        <f>X38/C38*C39*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A39-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A39-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y39" s="8">
+        <f>Q39-X39</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -19649,6 +20153,14 @@
         <f>Q40-V40</f>
         <v/>
       </c>
+      <c r="X40" s="8">
+        <f>X39/C39*C40*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A40-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A40-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y40" s="8">
+        <f>Q40-X40</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -19739,12 +20251,20 @@
         <f>Q41-V41</f>
         <v/>
       </c>
+      <c r="X41" s="8">
+        <f>X40/C40*C41*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A41-2026)/24))^Inputs!$B$32*(1+(Inputs!$B$35+(Inputs!$B$36-Inputs!$B$35)*(A41-2026)/24)+Inputs!$B$37)^Inputs!$B$33*(1+Inputs!$B$38)^Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="Y41" s="8">
+        <f>Q41-X41</f>
+        <v/>
+      </c>
     </row>
     <row r="42"/>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Every cell in columns F, H, K, O, P, Q, R, S, U, V and W is a live formula. Change any parameter on the Inputs sheet and this sheet recalculates.</t>
+          <t>Every cell in columns F, H, K, O, P, Q, R, S, U, V, W, X and Y is a live formula. Change any parameter on the Inputs sheet and this sheet recalculates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename the green line to "Revised projected need"
The label "World Bank demand" read as an external target rather than what
it is: the WHO per-head floor revised for what Tamil Nadu own economy
will support, anchored on the doctors the state has in 2025. Renamed in
every place it is displayed: chart legends, metric card, finding strip,
Compare options, the doctor table, workbook columns X and Y, Inputs rows
32 to 38, the Variables, Assumptions, Parameters, Methodology, Provenance
and Data Sources sheets, the CSV header, README and both documents. Code
identifiers follow (revised_need, rn_*), since Params field names show on
the Assumptions tab.

The method and its citation are unchanged: still the demand side of the
health labour market framework, Liu et al. 2017 Table 1, cited in full
wherever the basis is stated. All figures identical; engine verified at
0.000000 including the renamed series.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TN_Health_Workforce_Projections_2050.xlsx
+++ b/TN_Health_Workforce_Projections_2050.xlsx
@@ -12073,12 +12073,12 @@
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>World Bank demand (doctors)</t>
+          <t>Revised projected need (doctors)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>The number of doctors the economy would absorb, on the World Bank health labour market demand model. Rises with income, ageing and the shift away from out-of-pocket payment. A demand line, not a norm.</t>
+          <t>A need line revised for what the state's own economy will support: it starts from the doctors Tamil Nadu actually has in 2025 and rises with income, ageing and the shift away from out-of-pocket payment. The demand side of the health labour market framework, so a behavioural benchmark rather than a fixed per-head norm like the WHO floor.</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -12093,24 +12093,24 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. Code: build_wb_demand()</t>
+          <t>Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. Code: build_revised_need()</t>
         </is>
       </c>
     </row>
     <row r="18" ht="92" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Surplus vs WB demand</t>
+          <t>Surplus vs revised need</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>How far supply runs above what the economy would absorb.</t>
+          <t>How far supply runs above the revised projected need.</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Active doctors - World Bank demand.</t>
+          <t>Active doctors - revised projected need.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -12301,7 +12301,7 @@
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>World Bank demand line: growth paths of its three drivers</t>
+          <t>Revised projected need: growth paths of its three drivers</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -13156,7 +13156,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>A stock-and-flow supply model with an explicit education pipeline, following the WHO / World Bank Health Labour Market Framework as operationalised in Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. and in World Health Organization. Health Labour Market Analysis Guidebook. Geneva: WHO; 2021. The same three-lens structure, Supply, Need and Demand, used in the Centre's Andhra Pradesh projection. This round builds the Supply lens for Tamil Nadu to 2050, sets it against the WHO need floor, and adds the World Bank demand line from the same paper.</t>
+          <t>A stock-and-flow supply model with an explicit education pipeline, following the WHO / World Bank Health Labour Market Framework as operationalised in Liu JX, Goryakin Y, Maeda A, Bruckner T, Scheffler RM. Global Health Workforce Labor Market Projections for 2030. Human Resources for Health. 2017;15:11. doi:10.1186/s12960-017-0187-2. First issued as World Bank Policy Research Working Paper 7790, Washington DC: World Bank; 2016. and in World Health Organization. Health Labour Market Analysis Guidebook. Geneva: WHO; 2021. The same three-lens structure, Supply, Need and Demand, used in the Centre's Andhra Pradesh projection. This round builds the Supply lens for Tamil Nadu to 2050, sets it against the WHO need floor, and adds the revised projected need line, which is the demand side of the same paper.</t>
         </is>
       </c>
     </row>
@@ -13211,12 +13211,12 @@
     <row r="7" ht="74" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Module 6b, demand benchmark</t>
+          <t>Module 6b, revised projected need</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Doctors the economy would absorb, on the demand model of Liu et al. 2017: ln(physicians per 1,000) = -9.882 + 0.231 ln GDPpc(t-1) + 0.531 ln GDPpc(t-4) - 0.518 ln GDPpc(t-5) - 0.099 ln OOPpc(t-2) + 0.516 ln Pop65(t-3) + country effect, estimated by GLM with country fixed effects on 165 countries, 1990 to 2013. The country effect pins the level, so the line is anchored on Tamil Nadu's modelled 2025 density and moved by the three drivers, whose growth paths are assumptions marked for State confirmation. Result: 151,248 in 2025, 233,187 in 2040, 305,668 in 2050. Supply exceeds it throughout; the gap is 211,989 doctors in 2050.</t>
+          <t>A need line revised for the state's own economy, on the demand model of Liu et al. 2017: ln(physicians per 1,000) = -9.882 + 0.231 ln GDPpc(t-1) + 0.531 ln GDPpc(t-4) - 0.518 ln GDPpc(t-5) - 0.099 ln OOPpc(t-2) + 0.516 ln Pop65(t-3) + country effect, estimated by GLM with country fixed effects on 165 countries, 1990 to 2013. The country effect pins the level, so the line is anchored on Tamil Nadu's modelled 2025 density and moved by the three drivers, whose growth paths are assumptions marked for State confirmation. Result: 151,248 in 2025, 233,187 in 2040, 305,668 in 2050. Supply exceeds it throughout; the gap is 211,989 doctors in 2050.</t>
         </is>
       </c>
     </row>
@@ -14212,7 +14212,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>World Bank demand elasticities</t>
+          <t>Revised need elasticities</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -14234,7 +14234,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>World Bank demand driver paths</t>
+          <t>Revised need driver paths</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -15247,7 +15247,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>The principal method reference: the supply, need and demand framework, and the demand elasticities in Table 1 used for the World Bank demand line</t>
+          <t>The principal method reference: the supply, need and demand framework, and the demand elasticities in Table 1 used for the revised projected need line</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -16352,7 +16352,7 @@
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>WB demand: income elasticity</t>
+          <t>Revised need: income elasticity</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -16372,7 +16372,7 @@
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>WB demand: out-of-pocket elasticity</t>
+          <t>Revised need: out-of-pocket elasticity</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
@@ -16392,7 +16392,7 @@
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>WB demand: population 65+ elasticity</t>
+          <t>Revised need: population 65+ elasticity</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -16412,7 +16412,7 @@
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>WB demand: real GSDP per capita growth, 2026</t>
+          <t>Revised need: real GSDP per capita growth, 2026</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
@@ -16432,7 +16432,7 @@
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>WB demand: real GSDP per capita growth, 2050</t>
+          <t>Revised need: real GSDP per capita growth, 2050</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
@@ -16452,7 +16452,7 @@
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>WB demand: OOP growth less GDP growth</t>
+          <t>Revised need: OOP growth less GDP growth</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
@@ -16472,7 +16472,7 @@
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>WB demand: growth of population aged 65+</t>
+          <t>Revised need: growth of population aged 65+</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
@@ -16648,12 +16648,12 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>World Bank demand (doctors)</t>
+          <t>Revised projected need (doctors)</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Surplus vs WB demand</t>
+          <t>Surplus vs revised need</t>
         </is>
       </c>
     </row>

</xml_diff>